<commit_message>
Fix stale Aggregate Summary cache in BAF_Respondent_Tracker.xlsx
Respondents logged and all six dimension stats (avg/mean|gap|/max|gap|/
opposite-direction count) were still cached from the 5-respondent count;
recomputed for the current 6 (adds R-0LU91I).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BAF_Respondent_Tracker.xlsx
+++ b/BAF_Respondent_Tracker.xlsx
@@ -2604,7 +2604,7 @@
       </c>
       <c r="B4" s="14" t="n">
         <f aca="false">COUNTIFS('Respondent Log'!A3:A22,"&lt;&gt;",'Respondent Log'!C3:C22,"Y")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2636,11 +2636,11 @@
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE('Respondent Log'!W3:W22),"")</f>
-        <v>0.0140000000000001</v>
+        <v>-0.35</v>
       </c>
       <c r="C7" s="18" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(ABS(N('Respondent Log'!W3:W22)))/COUNT('Respondent Log'!W3:W22),"")</f>
-        <v>1.65</v>
+        <v>1.736667</v>
       </c>
       <c r="D7" s="18" t="n">
         <f aca="false">IFERROR(MAX(ABS(MIN('Respondent Log'!W3:W22)),ABS(MAX('Respondent Log'!W3:W22))),"")</f>
@@ -2648,11 +2648,11 @@
       </c>
       <c r="E7" s="19" t="n">
         <f aca="false">SUMPRODUCT(('Respondent Log'!W3:W22&lt;&gt;"")*(SIGN(N('Respondent Log'!K3:K22))&lt;&gt;SIGN(N('Respondent Log'!Q3:Q22)))*(N('Respondent Log'!K3:K22)&lt;&gt;0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">COUNT('Respondent Log'!W3:W22)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G7" s="19" t="str">
         <f aca="false">IF(F7=0,"",IF(OR(C7&gt;0.5,E7/MAX(F7,1)&gt;0.4),"REVIEW","ok"))</f>
@@ -2665,11 +2665,11 @@
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE('Respondent Log'!X3:X22),"")</f>
-        <v>0.032</v>
+        <v>0.225</v>
       </c>
       <c r="C8" s="18" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(ABS(N('Respondent Log'!X3:X22)))/COUNT('Respondent Log'!X3:X22),"")</f>
-        <v>0.756</v>
+        <v>0.828333</v>
       </c>
       <c r="D8" s="18" t="n">
         <f aca="false">IFERROR(MAX(ABS(MIN('Respondent Log'!X3:X22)),ABS(MAX('Respondent Log'!X3:X22))),"")</f>
@@ -2677,11 +2677,11 @@
       </c>
       <c r="E8" s="19" t="n">
         <f aca="false">SUMPRODUCT(('Respondent Log'!X3:X22&lt;&gt;"")*(SIGN(N('Respondent Log'!L3:L22))&lt;&gt;SIGN(N('Respondent Log'!R3:R22)))*(N('Respondent Log'!L3:L22)&lt;&gt;0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="19" t="n">
         <f aca="false">COUNT('Respondent Log'!X3:X22)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8" s="19" t="str">
         <f aca="false">IF(F8=0,"",IF(OR(C8&gt;0.5,E8/MAX(F8,1)&gt;0.4),"REVIEW","ok"))</f>
@@ -2694,11 +2694,11 @@
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE('Respondent Log'!Y3:Y22),"")</f>
-        <v>-0.502</v>
+        <v>-0.688333</v>
       </c>
       <c r="C9" s="18" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(ABS(N('Respondent Log'!Y3:Y22)))/COUNT('Respondent Log'!Y3:Y22),"")</f>
-        <v>1.39</v>
+        <v>1.428333</v>
       </c>
       <c r="D9" s="18" t="n">
         <f aca="false">IFERROR(MAX(ABS(MIN('Respondent Log'!Y3:Y22)),ABS(MAX('Respondent Log'!Y3:Y22))),"")</f>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="F9" s="19" t="n">
         <f aca="false">COUNT('Respondent Log'!Y3:Y22)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G9" s="19" t="str">
         <f aca="false">IF(F9=0,"",IF(OR(C9&gt;0.5,E9/MAX(F9,1)&gt;0.4),"REVIEW","ok"))</f>
@@ -2723,11 +2723,11 @@
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE('Respondent Log'!Z3:Z22),"")</f>
-        <v>-0.986</v>
+        <v>-0.628333</v>
       </c>
       <c r="C10" s="18" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(ABS(N('Respondent Log'!Z3:Z22)))/COUNT('Respondent Log'!Z3:Z22),"")</f>
-        <v>1.006</v>
+        <v>1.031667</v>
       </c>
       <c r="D10" s="18" t="n">
         <f aca="false">IFERROR(MAX(ABS(MIN('Respondent Log'!Z3:Z22)),ABS(MAX('Respondent Log'!Z3:Z22))),"")</f>
@@ -2735,11 +2735,11 @@
       </c>
       <c r="E10" s="19" t="n">
         <f aca="false">SUMPRODUCT(('Respondent Log'!Z3:Z22&lt;&gt;"")*(SIGN(N('Respondent Log'!N3:N22))&lt;&gt;SIGN(N('Respondent Log'!T3:T22)))*(N('Respondent Log'!N3:N22)&lt;&gt;0))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="19" t="n">
         <f aca="false">COUNT('Respondent Log'!Z3:Z22)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G10" s="19" t="str">
         <f aca="false">IF(F10=0,"",IF(OR(C10&gt;0.5,E10/MAX(F10,1)&gt;0.4),"REVIEW","ok"))</f>
@@ -2752,11 +2752,11 @@
       </c>
       <c r="B11" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE('Respondent Log'!AA3:AA22),"")</f>
-        <v>-0.214</v>
+        <v>-0.228333</v>
       </c>
       <c r="C11" s="18" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(ABS(N('Respondent Log'!AA3:AA22)))/COUNT('Respondent Log'!AA3:AA22),"")</f>
-        <v>1.098</v>
+        <v>0.965</v>
       </c>
       <c r="D11" s="18" t="n">
         <f aca="false">IFERROR(MAX(ABS(MIN('Respondent Log'!AA3:AA22)),ABS(MAX('Respondent Log'!AA3:AA22))),"")</f>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F11" s="19" t="n">
         <f aca="false">COUNT('Respondent Log'!AA3:AA22)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G11" s="19" t="str">
         <f aca="false">IF(F11=0,"",IF(OR(C11&gt;0.5,E11/MAX(F11,1)&gt;0.4),"REVIEW","ok"))</f>
@@ -2781,11 +2781,11 @@
       </c>
       <c r="B12" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE('Respondent Log'!AB3:AB22),"")</f>
-        <v>-0.218</v>
+        <v>-0.063333</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(ABS(N('Respondent Log'!AB3:AB22)))/COUNT('Respondent Log'!AB3:AB22),"")</f>
-        <v>0.662</v>
+        <v>0.67</v>
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">IFERROR(MAX(ABS(MIN('Respondent Log'!AB3:AB22)),ABS(MAX('Respondent Log'!AB3:AB22))),"")</f>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="F12" s="19" t="n">
         <f aca="false">COUNT('Respondent Log'!AB3:AB22)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G12" s="19" t="str">
         <f aca="false">IF(F12=0,"",IF(OR(C12&gt;0.5,E12/MAX(F12,1)&gt;0.4),"REVIEW","ok"))</f>

</xml_diff>